<commit_message>
Workflow: SetTransactionStatus, updated. Config file updated.
</commit_message>
<xml_diff>
--- a/Data/Config_Process_Name_Performer.xlsx
+++ b/Data/Config_Process_Name_Performer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PiotrDane\02 Firma\02 Nowy Kontrahent\03 PGajewski\My Templates\WindowsC_Performer_Template\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECEF973-1F34-437B-A395-E7D95797A733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1BEBE5E-820E-43EB-82AD-EEE6E940E648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="110">
   <si>
     <t>Name</t>
   </si>
@@ -300,15 +300,6 @@
     <t>EmailTo_Business</t>
   </si>
   <si>
-    <t>MultipleRobotRun</t>
-  </si>
-  <si>
-    <t>Boolean value specifying whether more than one Robot will be run at the same time. If set to true, output report will be saved with additional sufix with machine name &amp; user.</t>
-  </si>
-  <si>
-    <t>Excel report name without extension. Will be prefixed with today's date: yyyy-MM-dd_, can be sufixed with: _machine_user, if MultipleRobotRun selected.</t>
-  </si>
-  <si>
     <t>Outlook credential for prod environment.</t>
   </si>
   <si>
@@ -316,12 +307,6 @@
   </si>
   <si>
     <t>ExcelReportAccess</t>
-  </si>
-  <si>
-    <t>AssetNameForBlockRelease</t>
-  </si>
-  <si>
-    <t>Asset name for semaphore mechanism, used to indicate whether Robot can execute some operation, not getting conflicted with other Robot.</t>
   </si>
   <si>
     <t>EmailTo_Business, Process_Name_EmailToBusiness</t>
@@ -549,6 +534,27 @@
 "BE":["BE00: Missing input data: {0}, aborting process."],
 "Status": ["OK", "Error"]}</t>
   </si>
+  <si>
+    <t>BlockAssetB4UseReport</t>
+  </si>
+  <si>
+    <t>BlockAssetNameB4UseReport</t>
+  </si>
+  <si>
+    <t>Boolean value indicating whether to use asset semaphore mechanism, when executing operation on shared file.</t>
+  </si>
+  <si>
+    <t>Asset name for semaphore mechanism, used to indicate if Robot can execute operation on shared file.</t>
+  </si>
+  <si>
+    <t>AddExcelReportSufix</t>
+  </si>
+  <si>
+    <t>Boolean value indicating whether to add machine name &amp; user sufix to Excel report name, making it unique if multi-users run.</t>
+  </si>
+  <si>
+    <t>Excel report name without extension. Will be prefixed with today's date: yyyy-MM-dd_, can be sufixed with: _machine_user, if AddExcelReportSufix selected.</t>
+  </si>
 </sst>
 </file>
 
@@ -607,13 +613,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -983,10 +988,10 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:26">
@@ -1007,8 +1012,8 @@
       <c r="A6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>107</v>
+      <c r="B6" t="s">
+        <v>102</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -1019,10 +1024,10 @@
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:26">
@@ -1096,7 +1101,7 @@
         <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
@@ -1129,7 +1134,7 @@
         <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
         <v>83</v>
@@ -1176,7 +1181,7 @@
         <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1188,7 +1193,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z22"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="50.77734375" customWidth="1"/>
@@ -1235,7 +1240,7 @@
         <v>25</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
@@ -1389,30 +1394,41 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>92</v>
-      </c>
-      <c r="B21" s="3" t="b">
+        <v>107</v>
+      </c>
+      <c r="B21" t="b">
         <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" t="s">
-        <v>97</v>
+        <v>103</v>
+      </c>
+      <c r="B22" t="b">
+        <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>99</v>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B21" xr:uid="{B881C61D-E6BD-439D-A2DB-3DB7612D1F95}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B21:B22" xr:uid="{B881C61D-E6BD-439D-A2DB-3DB7612D1F95}">
       <formula1>"PRAWDA,FAŁSZ"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1483,17 +1499,17 @@
     </row>
     <row r="5" spans="1:26" ht="14.4">
       <c r="D5" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.4">
       <c r="D6" s="3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.4">
       <c r="D7" s="3" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.4"/>

</xml_diff>

<commit_message>
Config file updated. Sequence: End Process\Else If - Log Job Status & Send E-mail\boolAE, Workflow: If - NoSuccessStatus & Item was processed, added, to inform business about item status even if it's failed run.
</commit_message>
<xml_diff>
--- a/Data/Config_Process_Name_Performer.xlsx
+++ b/Data/Config_Process_Name_Performer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PiotrDane\02 Firma\02 Nowy Kontrahent\03 PGajewski\My Templates\WindowsC_Performer_Template\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A066453-BC4E-4350-B5F1-A4D9E31F1F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86D42B3-BBFE-4361-BAF4-10D961F45308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -324,6 +324,137 @@
     <t>ExcelReportFolder, Process_Name_OutputReportFolderPath</t>
   </si>
   <si>
+    <t>{"TO":{"Min":2, "VShort":4, "Short":8, "Medium":16, "Long":64, "VLong":256, "Max":512},
+"TOms":{"Min":2000, "VShort":4000, "Short":8000, "Medium":16000, "Long":64000, "VLong":256000, "Max":512000},
+"DEL":{"D1":1, "D2":2, "D3":3, "D4":4, "D6":6},
+"RS":{"ShowRobotStatus":{"NR":2, "TS":5}, "FoldersFilesCreateDelete":{"NR":3, "TS":4}, "AppXYLogin":{"NR":2, "TS":6}, "ExcelGetTable":{"NR":2, "TS":6}, "ExcelAddToReport":{"NR":2, "TS":4}, "OrchestratorGetSetActivities":{"NR":2, "TS":5}, "OutlookGetEmails":{"NR":2, "TS":8}, "OutlookSendEmail":{"NR":2, "TS":6}, "APIRunQuery":{"NR":2, "TS":6}, "SQLRunQuery":{"NR":2, "TS":6}, "AssetBlockAndRelease":{"NR":15, "TS":2}},
+"SE":["SE00: Critical error while initializing the environment."], 
+"AE":["AE00: Unexpected application exception.", 
+"AE01: Robot couldn't login to AppXY.", 
+"AE02: Robot couldn't logout from AppXY."], 
+"BE":["BE00: Missing input data: {0}, aborting process."],
+"Status": ["OK", "Error"]}</t>
+  </si>
+  <si>
+    <t>BlockAssetB4UseReport</t>
+  </si>
+  <si>
+    <t>BlockAssetNameB4UseReport</t>
+  </si>
+  <si>
+    <t>Boolean value indicating whether to use asset semaphore mechanism, when executing operation on shared file.</t>
+  </si>
+  <si>
+    <t>Asset name for semaphore mechanism, used to indicate if Robot can execute operation on shared file.</t>
+  </si>
+  <si>
+    <t>AddExcelReportSufix</t>
+  </si>
+  <si>
+    <t>Boolean value indicating whether to add machine name &amp; user sufix to Excel report name, making it unique if multi-users run.</t>
+  </si>
+  <si>
+    <t>Excel report name without extension. Will be prefixed with today's date: yyyy-MM-dd_, can be sufixed with: _machine_user, if AddExcelReportSufix selected.</t>
+  </si>
+  <si>
+    <t>ColNo_Width</t>
+  </si>
+  <si>
+    <t>Dictionary where key is report column number, value is corresponding desired width in px.</t>
+  </si>
+  <si>
+    <t>&lt;!DOCTYPE html&gt;
+&lt;html&gt;
+&lt;head&gt;
+&lt;meta http-equiv="Content-Type" content="text/html; charset=UTF-8"&gt;
+&lt;meta name="viewport" content="width=device-width, initial-scale=1.0"&gt;
+&lt;style&gt;
+body {
+  background-color: white;
+}
+#tableMain {
+  width: 900px;
+  margin-top: 30px;
+  margin-left: 20px;
+  background-color: #EDEDED;
+  font-family: Verdana, Arial, sans-serif;
+  color: #333;
+  border: 2px solid #ddd;
+  border-collapse: collapse;
+  white-space: normal;
+}
+#tableMainHeader {
+  background-color: #27CCF5;
+  padding: 14px;
+  font-size: 16px;
+  font-weight: bold;
+}
+#tableSecondRow {
+  padding: 12px 12px 10px;
+  font-size: 12px;
+  color: #006400;
+}
+.tableHeader th {
+  background-color: #f8f8f8;
+  font-weight: bold;
+  padding: 12px;
+  font-size: 12px;
+  border-bottom: 1px solid #ddd;
+  text-align: left;
+}
+.tableContent td {
+  background-color: #f8f8f8;
+  padding: 12px;
+  font-size: 12px;
+  border-bottom: 1px solid #ddd;
+  color: #006400;
+  text-align: left;
+}
+#tableFooter {
+  padding: 10px;
+  font-size: 11px;
+  color: #777;
+  text-align: center;
+  border-bottom: 1px solid #ddd;
+}
+&lt;/style&gt;
+&lt;/head&gt;
+&lt;body&gt;
+&lt;table id="tableMain"&gt;
+&lt;!--Main Header--&gt;
+&lt;tr&gt;
+&lt;td id="tableMainHeader" colspan="&lt;varColSpan&gt;"&gt;
+📈 Robot report: &lt;varProcessName&gt;
+&lt;/td&gt;
+&lt;/tr&gt;
+&lt;!--Row2--&gt;
+&lt;tr&gt;
+&lt;td id="tableSecondRow" colspan="&lt;varColSpan&gt;"&gt;
+&lt;varDesc&gt;
+&lt;/td&gt;
+&lt;/tr&gt;
+&lt;!--Header--&gt;
+&lt;tr class="tableHeader"&gt;
+&lt;varTableHeader&gt;
+&lt;/tr&gt;
+&lt;!--Content--&gt;
+&lt;tbody class="tableContent"&gt;
+&lt;varTableContent&gt;
+&lt;/tbody&gt;
+&lt;!--Footer--&gt;
+&lt;tr&gt;
+&lt;td id="tableFooter" colspan="&lt;varColSpan&gt;"&gt;
+This is an automatic message – please do not reply.
+&lt;/td&gt;
+&lt;/tr&gt;
+&lt;/table&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
+  </si>
+  <si>
+    <t>{1:150, 2:100, 3:300, 4:150, 5:100, 6:100}</t>
+  </si>
+  <si>
     <t>&lt;!DOCTYPE html&gt;
 &lt;html&gt;
 &lt;head&gt;
@@ -337,7 +468,6 @@
   padding: 12px;
 }
 #tableMain {
-  width: 90%;
   max-width: 600px;
   margin-top: 30px;
   margin-left: 20px;
@@ -433,137 +563,6 @@
 &lt;/body&gt;
 &lt;/html&gt;</t>
   </si>
-  <si>
-    <t>&lt;!DOCTYPE html&gt;
-&lt;html&gt;
-&lt;head&gt;
-&lt;meta http-equiv="Content-Type" content="text/html; charset=UTF-8"&gt;
-&lt;meta name="viewport" content="width=device-width, initial-scale=1.0"&gt;
-&lt;style&gt;
-body {
-  background-color: white;
-}
-#tableMain {
-  width: 1000px;
-  margin-top: 30px;
-  margin-left: 20px;
-  background-color: #EDEDED;
-  font-family: Verdana, Arial, sans-serif;
-  color: #333;
-  border: 2px solid #ddd;
-  border-collapse: collapse;
-  white-space: normal;
-}
-#tableMainHeader {
-  background-color: #27CCF5;
-  padding: 14px;
-  font-size: 16px;
-  font-weight: bold;
-}
-#tableSecondRow {
-  padding: 12px 12px 10px;
-  font-size: 12px;
-  color: #006400;
-}
-.tableHeader th {
-  background-color: #f8f8f8;
-  font-weight: bold;
-  padding: 12px;
-  font-size: 12px;
-  border-bottom: 1px solid #ddd;
-  text-align: left;
-}
-.tableContent td {
-  background-color: #f8f8f8;
-  padding: 12px;
-  font-size: 12px;
-  border-bottom: 1px solid #ddd;
-  color: #006400;
-  text-align: left;
-}
-#tableFooter {
-  padding: 10px;
-  font-size: 11px;
-  color: #777;
-  text-align: center;
-  border-bottom: 1px solid #ddd;
-}
-&lt;/style&gt;
-&lt;/head&gt;
-&lt;body&gt;
-&lt;table id="tableMain"&gt;
-&lt;!--Main Header--&gt;
-&lt;tr&gt;
-&lt;td id="tableMainHeader" colspan="&lt;varColSpan&gt;"&gt;
-📈 Robot report: &lt;varProcessName&gt;
-&lt;/td&gt;
-&lt;/tr&gt;
-&lt;!--Row2--&gt;
-&lt;tr&gt;
-&lt;td id="tableSecondRow" colspan="&lt;varColSpan&gt;"&gt;
-&lt;varDesc&gt;
-&lt;/td&gt;
-&lt;/tr&gt;
-&lt;!--Header--&gt;
-&lt;tr class="tableHeader"&gt;
-&lt;varTableHeader&gt;
-&lt;/tr&gt;
-&lt;!--Content--&gt;
-&lt;tbody class="tableContent"&gt;
-&lt;varTableContent&gt;
-&lt;/tbody&gt;
-&lt;!--Footer--&gt;
-&lt;tr&gt;
-&lt;td id="tableFooter" colspan="&lt;varColSpan&gt;"&gt;
-This is an automatic message – please do not reply.
-&lt;/td&gt;
-&lt;/tr&gt;
-&lt;/table&gt;
-&lt;/body&gt;
-&lt;/html&gt;</t>
-  </si>
-  <si>
-    <t>{"TO":{"Min":2, "VShort":4, "Short":8, "Medium":16, "Long":64, "VLong":256, "Max":512},
-"TOms":{"Min":2000, "VShort":4000, "Short":8000, "Medium":16000, "Long":64000, "VLong":256000, "Max":512000},
-"DEL":{"D1":1, "D2":2, "D3":3, "D4":4, "D6":6},
-"RS":{"ShowRobotStatus":{"NR":2, "TS":5}, "FoldersFilesCreateDelete":{"NR":3, "TS":4}, "AppXYLogin":{"NR":2, "TS":6}, "ExcelGetTable":{"NR":2, "TS":6}, "ExcelAddToReport":{"NR":2, "TS":4}, "OrchestratorGetSetActivities":{"NR":2, "TS":5}, "OutlookGetEmails":{"NR":2, "TS":8}, "OutlookSendEmail":{"NR":2, "TS":6}, "APIRunQuery":{"NR":2, "TS":6}, "SQLRunQuery":{"NR":2, "TS":6}, "AssetBlockAndRelease":{"NR":15, "TS":2}},
-"SE":["SE00: Critical error while initializing the environment."], 
-"AE":["AE00: Unexpected application exception.", 
-"AE01: Robot couldn't login to AppXY.", 
-"AE02: Robot couldn't logout from AppXY."], 
-"BE":["BE00: Missing input data: {0}, aborting process."],
-"Status": ["OK", "Error"]}</t>
-  </si>
-  <si>
-    <t>BlockAssetB4UseReport</t>
-  </si>
-  <si>
-    <t>BlockAssetNameB4UseReport</t>
-  </si>
-  <si>
-    <t>Boolean value indicating whether to use asset semaphore mechanism, when executing operation on shared file.</t>
-  </si>
-  <si>
-    <t>Asset name for semaphore mechanism, used to indicate if Robot can execute operation on shared file.</t>
-  </si>
-  <si>
-    <t>AddExcelReportSufix</t>
-  </si>
-  <si>
-    <t>Boolean value indicating whether to add machine name &amp; user sufix to Excel report name, making it unique if multi-users run.</t>
-  </si>
-  <si>
-    <t>Excel report name without extension. Will be prefixed with today's date: yyyy-MM-dd_, can be sufixed with: _machine_user, if AddExcelReportSufix selected.</t>
-  </si>
-  <si>
-    <t>ColNo_Width</t>
-  </si>
-  <si>
-    <t>{1:150, 2:250, 3:150, 4:150, 5:150, 6:150}</t>
-  </si>
-  <si>
-    <t>Dictionary where key is report column number, value is corresponding desired width in px.</t>
-  </si>
 </sst>
 </file>
 
@@ -622,12 +621,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -1022,7 +1022,7 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -1110,7 +1110,7 @@
         <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
@@ -1118,13 +1118,13 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B17" t="s">
         <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1153,8 +1153,8 @@
       <c r="A21" t="s">
         <v>82</v>
       </c>
-      <c r="B21" t="s">
-        <v>100</v>
+      <c r="B21" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="C21" t="s">
         <v>83</v>
@@ -1201,7 +1201,7 @@
         <v>44</v>
       </c>
       <c r="C26" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1414,35 +1414,35 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B21" t="b">
         <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B22" t="b">
         <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B23" t="s">
         <v>94</v>
       </c>
       <c r="C23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>